<commit_message>
Actually add the TEKTA figures, which the previous commit only claimed
The previous commit message said the TEKTA network figures had been added to
comparables_data.py. They had not: the edit used a string match that did not
correspond to the file's actual characters, and it failed silently. The workbook
shipped without them.

Now genuinely added and verified present in the Comparables sheet: 45,000
Division I athletes, 68 Power Four universities, and the claimed 50-70%
speed-to-market gain, plus the press release in the source links. Inserted with
a line-based edit rather than a fragile string match, and checked by reading the
figures back out of the generated workbook rather than trusting the write.

The three rows are marked as an agency's addressable supply rather than a user
base, so nothing in the model treats them as comparable to Patreon members or
OnlyFans creator accounts.

All 3,592 formula references still resolve.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/business-plan/Stride_Financial_Model.xlsx
+++ b/business-plan/Stride_Financial_Model.xlsx
@@ -2256,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2853,112 +2853,139 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="58" t="inlineStr">
+        <is>
+          <t>Division I athletes in network</t>
+        </is>
+      </c>
+      <c r="B23" s="59" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C23" s="60" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D23" s="60" t="inlineStr">
+        <is>
+          <t>TEKTA</t>
+        </is>
+      </c>
+      <c r="E23" s="60" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F23" s="60" t="inlineStr">
+        <is>
+          <t>Publicis Groupe press release, 19 Aug 2026</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="62" t="inlineStr">
+      <c r="A24" s="58" t="inlineStr">
+        <is>
+          <t>Power Four universities</t>
+        </is>
+      </c>
+      <c r="B24" s="59" t="n">
+        <v>68</v>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D24" s="60" t="inlineStr">
+        <is>
+          <t>TEKTA</t>
+        </is>
+      </c>
+      <c r="E24" s="60" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F24" s="60" t="inlineStr">
+        <is>
+          <t>Publicis Groupe press release</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="58" t="inlineStr">
+        <is>
+          <t>Claimed speed-to-market gain</t>
+        </is>
+      </c>
+      <c r="B25" s="61" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C25" s="60" t="inlineStr">
+        <is>
+          <t>share faster</t>
+        </is>
+      </c>
+      <c r="D25" s="60" t="inlineStr">
+        <is>
+          <t>TEKTA</t>
+        </is>
+      </c>
+      <c r="E25" s="60" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+      <c r="F25" s="60" t="inlineStr">
+        <is>
+          <t>Publicis — stated 50-70% vs a traditional agency process</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="62" t="inlineStr">
         <is>
           <t>TAKE RATES - what each platform costs a creator</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Headline take</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>Per txn (USD)</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Monthly fee (USD)</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr"/>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>OnlyFans</t>
-        </is>
-      </c>
-      <c r="B26" s="63" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C26" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="65" t="inlineStr">
-        <is>
-          <t>Company disclosure — 80% creator share</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Fansly</t>
-        </is>
-      </c>
-      <c r="B27" s="63" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C27" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="65" t="inlineStr">
-        <is>
-          <t>MEXC platform comparison 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Fanfix</t>
-        </is>
-      </c>
-      <c r="B28" s="63" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C28" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="65" t="inlineStr">
-        <is>
-          <t>Outseeker comparison 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Patreon</t>
+          <t>OnlyFans</t>
         </is>
       </c>
       <c r="B29" s="63" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C29" s="64" t="n">
         <v>0</v>
@@ -2968,39 +2995,39 @@
       </c>
       <c r="F29" s="65" t="inlineStr">
         <is>
-          <t>8-12% by plan tier; 10% midpoint</t>
+          <t>Company disclosure — 80% creator share</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Passes</t>
+          <t>Fansly</t>
         </is>
       </c>
       <c r="B30" s="63" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C30" s="64" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D30" s="64" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F30" s="65" t="inlineStr">
         <is>
-          <t>Sacra; Passes rebrand release Apr 2026</t>
+          <t>MEXC platform comparison 2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Stride (proposed)</t>
+          <t>Fanfix</t>
         </is>
       </c>
       <c r="B31" s="63" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="C31" s="64" t="n">
         <v>0</v>
@@ -3010,222 +3037,299 @@
       </c>
       <c r="F31" s="65" t="inlineStr">
         <is>
+          <t>Outseeker comparison 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Patreon</t>
+        </is>
+      </c>
+      <c r="B32" s="63" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C32" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="65" t="inlineStr">
+        <is>
+          <t>8-12% by plan tier; 10% midpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Passes</t>
+        </is>
+      </c>
+      <c r="B33" s="63" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C33" s="64" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D33" s="64" t="n">
+        <v>29</v>
+      </c>
+      <c r="F33" s="65" t="inlineStr">
+        <is>
+          <t>Sacra; Passes rebrand release Apr 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Stride (proposed)</t>
+        </is>
+      </c>
+      <c r="B34" s="63" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C34" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="65" t="inlineStr">
+        <is>
           <t>Our decision — see MarketModel</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="62" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
         <is>
           <t>INTERMEDIARIES the athlete already pays</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>Sports agent — endorsement</t>
         </is>
       </c>
-      <c r="B34" s="63" t="n">
+      <c r="B37" s="63" t="n">
         <v>0.1</v>
       </c>
-      <c r="C34" s="63" t="n">
+      <c r="C37" s="63" t="n">
         <v>0.2</v>
       </c>
-      <c r="F34" s="65" t="inlineStr">
+      <c r="F37" s="65" t="inlineStr">
         <is>
           <t>Oreate / Sapling agent-commission surveys</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Sports agent — playing contract</t>
         </is>
       </c>
-      <c r="B35" s="63" t="n">
+      <c r="B38" s="63" t="n">
         <v>0.04</v>
       </c>
-      <c r="C35" s="63" t="n">
+      <c r="C38" s="63" t="n">
         <v>0.1</v>
       </c>
-      <c r="F35" s="65" t="inlineStr">
+      <c r="F38" s="65" t="inlineStr">
         <is>
           <t>Same</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>OnlyFans management agency</t>
         </is>
       </c>
-      <c r="B36" s="63" t="n">
+      <c r="B39" s="63" t="n">
         <v>0.2</v>
       </c>
-      <c r="C36" s="63" t="n">
+      <c r="C39" s="63" t="n">
         <v>0.5</v>
       </c>
-      <c r="F36" s="65" t="inlineStr">
+      <c r="F39" s="65" t="inlineStr">
         <is>
           <t>Aruna Talent rate guide 2026 — on top of the 20%</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>SOURCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="66" t="inlineStr">
-        <is>
-          <t>OnlyFans FY2024</t>
-        </is>
-      </c>
-      <c r="B40" s="67" t="inlineStr">
-        <is>
-          <t>https://variety.com/2025/digital/news/onlyfans-fiscal-2024-revenue-earnings-1236495750/</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="66" t="inlineStr">
-        <is>
-          <t>Patreon creators</t>
-        </is>
-      </c>
-      <c r="B41" s="67" t="inlineStr">
-        <is>
-          <t>https://backlinko.com/patreon-users</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="66" t="inlineStr">
-        <is>
-          <t>Passes economics</t>
-        </is>
-      </c>
-      <c r="B42" s="67" t="inlineStr">
-        <is>
-          <t>https://sacra.com/c/passes/</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="66" t="inlineStr">
         <is>
-          <t>Platform comparison</t>
+          <t>OnlyFans FY2024</t>
         </is>
       </c>
       <c r="B43" s="67" t="inlineStr">
         <is>
-          <t>https://www.mexc.com/news/1014749</t>
+          <t>https://variety.com/2025/digital/news/onlyfans-fiscal-2024-revenue-earnings-1236495750/</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="66" t="inlineStr">
         <is>
-          <t>Agency commissions</t>
+          <t>Patreon creators</t>
         </is>
       </c>
       <c r="B44" s="67" t="inlineStr">
         <is>
-          <t>https://arunatalent.com/blog/onlyfans-agency-commission-rates/</t>
+          <t>https://backlinko.com/patreon-users</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="66" t="inlineStr">
         <is>
-          <t>Agent commissions</t>
+          <t>Passes economics</t>
         </is>
       </c>
       <c r="B45" s="67" t="inlineStr">
         <is>
-          <t>https://www.oreateai.com/blog/understanding-sports-agents-commission-what-percentage-do-they-take/95c2df506ae450b9b71340b89cfcfece</t>
+          <t>https://sacra.com/c/passes/</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="66" t="inlineStr">
         <is>
-          <t>Eurobarometer 525</t>
+          <t>Platform comparison</t>
         </is>
       </c>
       <c r="B46" s="67" t="inlineStr">
         <is>
-          <t>https://europa.eu/eurobarometer/surveys/detail/2668</t>
+          <t>https://www.mexc.com/news/1014749</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="66" t="inlineStr">
         <is>
-          <t>FIP World Padel Report 2025</t>
+          <t>Agency commissions</t>
         </is>
       </c>
       <c r="B47" s="67" t="inlineStr">
         <is>
-          <t>https://www.padelfip.com/2025/12/online-the-fip-world-padel-report-2025-a-comprehensive-analysis-of-a-sport-in-constant-growth/</t>
+          <t>https://arunatalent.com/blog/onlyfans-agency-commission-rates/</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="66" t="inlineStr">
         <is>
-          <t>Stripe EU pricing</t>
+          <t>Agent commissions</t>
         </is>
       </c>
       <c r="B48" s="67" t="inlineStr">
         <is>
-          <t>https://stripe.com/es/pricing</t>
+          <t>https://www.oreateai.com/blog/understanding-sports-agents-commission-what-percentage-do-they-take/95c2df506ae450b9b71340b89cfcfece</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="66" t="inlineStr">
         <is>
+          <t>Eurobarometer 525</t>
+        </is>
+      </c>
+      <c r="B49" s="67" t="inlineStr">
+        <is>
+          <t>https://europa.eu/eurobarometer/surveys/detail/2668</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="66" t="inlineStr">
+        <is>
+          <t>FIP World Padel Report 2025</t>
+        </is>
+      </c>
+      <c r="B50" s="67" t="inlineStr">
+        <is>
+          <t>https://www.padelfip.com/2025/12/online-the-fip-world-padel-report-2025-a-comprehensive-analysis-of-a-sport-in-constant-growth/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="66" t="inlineStr">
+        <is>
+          <t>Stripe EU pricing</t>
+        </is>
+      </c>
+      <c r="B51" s="67" t="inlineStr">
+        <is>
+          <t>https://stripe.com/es/pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="66" t="inlineStr">
+        <is>
+          <t>TEKTA launch</t>
+        </is>
+      </c>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>https://www.publicisgroupe.com/en/news/press-releases/publicis-sports-and-travis-kelce-s-tekta-join-forces-to-reimagine-the-future-of-nil-marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="66" t="inlineStr">
+        <is>
           <t>Stripe Connect age</t>
         </is>
       </c>
-      <c r="B49" s="67" t="inlineStr">
+      <c r="B53" s="67" t="inlineStr">
         <is>
           <t>https://support.stripe.com/questions/age-requirement-to-create-a-stripe-account</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B53:F53"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B51:F51"/>
     <mergeCell ref="B45:F45"/>
     <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B52:F52"/>
     <mergeCell ref="B49:F49"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3866,7 +3970,7 @@
         </is>
       </c>
       <c r="B47" s="28">
-        <f>B46*(1-Comparables!B26)-B46/Assumptions!$C$44*Comparables!C26*B45-Comparables!D26*B45</f>
+        <f>B46*(1-Comparables!B29)-B46/Assumptions!$C$44*Comparables!C29*B45-Comparables!D29*B45</f>
         <v/>
       </c>
       <c r="D47" s="68" t="inlineStr">
@@ -3882,7 +3986,7 @@
         </is>
       </c>
       <c r="B48" s="28">
-        <f>B46*(1-Comparables!B29)-B46/Assumptions!$C$44*Comparables!C29*B45-Comparables!D29*B45</f>
+        <f>B46*(1-Comparables!B32)-B46/Assumptions!$C$44*Comparables!C32*B45-Comparables!D32*B45</f>
         <v/>
       </c>
       <c r="D48" s="68" t="inlineStr">
@@ -3898,7 +4002,7 @@
         </is>
       </c>
       <c r="B49" s="28">
-        <f>B46*(1-Comparables!B30)-B46/Assumptions!$C$44*Comparables!C30*B45-Comparables!D30*B45</f>
+        <f>B46*(1-Comparables!B33)-B46/Assumptions!$C$44*Comparables!C33*B45-Comparables!D33*B45</f>
         <v/>
       </c>
       <c r="D49" s="68" t="inlineStr">
@@ -3914,7 +4018,7 @@
         </is>
       </c>
       <c r="B50" s="28">
-        <f>B46*(1-Comparables!B31)-B46/Assumptions!$C$44*Comparables!C31*B45-Comparables!D31*B45</f>
+        <f>B46*(1-Comparables!B34)-B46/Assumptions!$C$44*Comparables!C34*B45-Comparables!D34*B45</f>
         <v/>
       </c>
       <c r="D50" s="68" t="inlineStr">
@@ -3930,7 +4034,7 @@
         </is>
       </c>
       <c r="B51" s="29">
-        <f>Comparables!D30*B45/((Comparables!B31-Comparables!B30)-Comparables!C30*B45/Assumptions!$C$44)</f>
+        <f>Comparables!D33*B45/((Comparables!B34-Comparables!B33)-Comparables!C33*B45/Assumptions!$C$44)</f>
         <v/>
       </c>
       <c r="D51" s="68" t="inlineStr">

</xml_diff>